<commit_message>
using 2022 HM64 rural urban interstate pavement for SC
</commit_message>
<xml_diff>
--- a/AHR 29th/AHR_data 29th dashboard.xlsx
+++ b/AHR 29th/AHR_data 29th dashboard.xlsx
@@ -5811,13 +5811,13 @@
         <v>1.731385488861424</v>
       </c>
       <c r="E202">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
       <c r="F202">
-        <v>0.7854922820323976</v>
+        <v>0.7901388763690342</v>
       </c>
       <c r="G202">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="203">
@@ -5838,13 +5838,13 @@
         <v>10.85917412642226</v>
       </c>
       <c r="E203">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
       <c r="F203">
-        <v>4.926573267724375</v>
+        <v>4.955716504352496</v>
       </c>
       <c r="G203">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="204">
@@ -5865,13 +5865,13 @@
         <v>5.158633032912483</v>
       </c>
       <c r="E204">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
       <c r="F204">
-        <v>2.340360629829937</v>
+        <v>2.354205077060045</v>
       </c>
       <c r="G204">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="205">
@@ -5892,13 +5892,13 @@
         <v>2.399072717960698</v>
       </c>
       <c r="E205">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
       <c r="F205">
-        <v>1.088407588094001</v>
+        <v>1.094846083608819</v>
       </c>
       <c r="G205">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="206">
@@ -5919,13 +5919,13 @@
         <v>7.292500101914317</v>
       </c>
       <c r="E206">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
       <c r="F206">
-        <v>3.308450130618278</v>
+        <v>3.328021329459594</v>
       </c>
       <c r="G206">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="207">
@@ -5946,13 +5946,13 @@
         <v>7.208684798054684</v>
       </c>
       <c r="E207">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
       <c r="F207">
-        <v>3.270424933617674</v>
+        <v>3.28977119369247</v>
       </c>
       <c r="G207">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="208">
@@ -5973,10 +5973,10 @@
         <v>0.03388681802778719</v>
       </c>
       <c r="E208">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
       <c r="F208">
-        <v>0.01537371902138749</v>
+        <v>0.01546466254479549</v>
       </c>
       <c r="G208">
         <v>1</v>
@@ -5997,7 +5997,7 @@
         </is>
       </c>
       <c r="E209">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
     </row>
     <row r="210">
@@ -6018,10 +6018,10 @@
         <v>0.1733549512754773</v>
       </c>
       <c r="E210">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
       <c r="F210">
-        <v>0.07864740530344617</v>
+        <v>0.07911264550558872</v>
       </c>
       <c r="G210">
         <v>2</v>
@@ -6045,10 +6045,10 @@
         <v>0.7580686936581237</v>
       </c>
       <c r="E211">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
       <c r="F211">
-        <v>0.3439194286596548</v>
+        <v>0.3459538904946386</v>
       </c>
       <c r="G211">
         <v>16</v>
@@ -6069,7 +6069,7 @@
         </is>
       </c>
       <c r="E212">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
     </row>
     <row r="213">
@@ -6090,10 +6090,10 @@
         <v>1.058758503352351</v>
       </c>
       <c r="E213">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
       <c r="F213">
-        <v>0.4803359149477122</v>
+        <v>0.4831773510676245</v>
       </c>
       <c r="G213">
         <v>22</v>
@@ -6117,10 +6117,10 @@
         <v>1.325808474424438</v>
       </c>
       <c r="E214">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
       <c r="F214">
-        <v>0.6014907314479032</v>
+        <v>0.60504886115868</v>
       </c>
       <c r="G214">
         <v>25</v>
@@ -6144,13 +6144,13 @@
         <v>2.14079563327743</v>
       </c>
       <c r="E215">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
       <c r="F215">
-        <v>0.9712328410779868</v>
+        <v>0.9769781871776732</v>
       </c>
       <c r="G215">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="216">
@@ -6171,13 +6171,13 @@
         <v>1.758128336987306</v>
       </c>
       <c r="E216">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
       <c r="F216">
-        <v>0.7976249358738358</v>
+        <v>0.8023433011519795</v>
       </c>
       <c r="G216">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="217">
@@ -6198,10 +6198,10 @@
         <v>0.6238174877539552</v>
       </c>
       <c r="E217">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
       <c r="F217">
-        <v>0.2830125498798091</v>
+        <v>0.2846867159302585</v>
       </c>
       <c r="G217">
         <v>13</v>
@@ -6225,10 +6225,10 @@
         <v>1.244698090608046</v>
       </c>
       <c r="E218">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
       <c r="F218">
-        <v>0.5646926983753501</v>
+        <v>0.5680331486308534</v>
       </c>
       <c r="G218">
         <v>24</v>
@@ -6252,13 +6252,13 @@
         <v>4.549685709612211</v>
       </c>
       <c r="E219">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
       <c r="F219">
-        <v>2.064094353085754</v>
+        <v>2.076304541970763</v>
       </c>
       <c r="G219">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="220">
@@ -6279,10 +6279,10 @@
         <v>0.1933543397307362</v>
       </c>
       <c r="E220">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
       <c r="F220">
-        <v>0.08772069682519988</v>
+        <v>0.08823961025362868</v>
       </c>
       <c r="G220">
         <v>3</v>
@@ -6306,13 +6306,13 @@
         <v>1.51333933697304</v>
       </c>
       <c r="E221">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
       <c r="F221">
-        <v>0.6865694421812787</v>
+        <v>0.6906308566021727</v>
       </c>
       <c r="G221">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="222">
@@ -6333,13 +6333,13 @@
         <v>2.014122818366372</v>
       </c>
       <c r="E222">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
       <c r="F222">
-        <v>0.9137641149646667</v>
+        <v>0.9191695037364453</v>
       </c>
       <c r="G222">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="223">
@@ -6360,13 +6360,13 @@
         <v>2.298412986503718</v>
       </c>
       <c r="E223">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
       <c r="F223">
-        <v>1.042740437318175</v>
+        <v>1.048908787945489</v>
       </c>
       <c r="G223">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="224">
@@ -6387,10 +6387,10 @@
         <v>0.5061183343323008</v>
       </c>
       <c r="E224">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
       <c r="F224">
-        <v>0.2296149805867606</v>
+        <v>0.2309732723138808</v>
       </c>
       <c r="G224">
         <v>9</v>
@@ -6414,13 +6414,13 @@
         <v>1.813524357899032</v>
       </c>
       <c r="E225">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
       <c r="F225">
-        <v>0.8227569166842332</v>
+        <v>0.8276239506665428</v>
       </c>
       <c r="G225">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="226">
@@ -6441,10 +6441,10 @@
         <v>1.120792126283758</v>
       </c>
       <c r="E226">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
       <c r="F226">
-        <v>0.5084792327429719</v>
+        <v>0.5114871511875014</v>
       </c>
       <c r="G226">
         <v>23</v>
@@ -6468,13 +6468,13 @@
         <v>1.492604821565878</v>
       </c>
       <c r="E227">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
       <c r="F227">
-        <v>0.6771626394046668</v>
+        <v>0.681168407707187</v>
       </c>
       <c r="G227">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="228">
@@ -6495,10 +6495,10 @@
         <v>0.5662787055109763</v>
       </c>
       <c r="E228">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
       <c r="F228">
-        <v>0.2569084444335262</v>
+        <v>0.2584281911582811</v>
       </c>
       <c r="G228">
         <v>12</v>
@@ -6522,10 +6522,10 @@
         <v>0.5323273346692246</v>
       </c>
       <c r="E229">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
       <c r="F229">
-        <v>0.2415054391916645</v>
+        <v>0.2429340691498245</v>
       </c>
       <c r="G229">
         <v>10</v>
@@ -6549,10 +6549,10 @@
         <v>0.3884581319825349</v>
       </c>
       <c r="E230">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
       <c r="F230">
-        <v>0.1762350825555669</v>
+        <v>0.1772776044940391</v>
       </c>
       <c r="G230">
         <v>5</v>
@@ -6576,10 +6576,10 @@
         <v>0.9135472370766489</v>
       </c>
       <c r="E231">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
       <c r="F231">
-        <v>0.414456692985003</v>
+        <v>0.4169084193309607</v>
       </c>
       <c r="G231">
         <v>17</v>
@@ -6603,13 +6603,13 @@
         <v>2.894558860284633</v>
       </c>
       <c r="E232">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
       <c r="F232">
-        <v>1.313198972308154</v>
+        <v>1.32096722547522</v>
       </c>
       <c r="G232">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="233">
@@ -6630,13 +6630,13 @@
         <v>2.081965796822538</v>
       </c>
       <c r="E233">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
       <c r="F233">
-        <v>0.9445430121601446</v>
+        <v>0.9501304740759474</v>
       </c>
       <c r="G233">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="234">
@@ -6657,10 +6657,10 @@
         <v>1.016120503452046</v>
       </c>
       <c r="E234">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
       <c r="F234">
-        <v>0.4609919733134247</v>
+        <v>0.4637189799835486</v>
       </c>
       <c r="G234">
         <v>20</v>
@@ -6684,10 +6684,10 @@
         <v>0.4708121204987101</v>
       </c>
       <c r="E235">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
       <c r="F235">
-        <v>0.2135973122786426</v>
+        <v>0.2148608511882634</v>
       </c>
       <c r="G235">
         <v>7</v>
@@ -6711,10 +6711,10 @@
         <v>0.9524788273159156</v>
       </c>
       <c r="E236">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
       <c r="F236">
-        <v>0.4321191164354282</v>
+        <v>0.4346753251787988</v>
       </c>
       <c r="G236">
         <v>19</v>
@@ -6738,13 +6738,13 @@
         <v>1.714992322092129</v>
       </c>
       <c r="E237">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
       <c r="F237">
-        <v>0.7780550555694339</v>
+        <v>0.7826576548533456</v>
       </c>
       <c r="G237">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="238">
@@ -6765,10 +6765,10 @@
         <v>0.6886384748980169</v>
       </c>
       <c r="E238">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
       <c r="F238">
-        <v>0.3124204347459719</v>
+        <v>0.31426856369128</v>
       </c>
       <c r="G238">
         <v>15</v>
@@ -6792,13 +6792,13 @@
         <v>2.671462200005628</v>
       </c>
       <c r="E239">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
       <c r="F239">
-        <v>1.211984825647145</v>
+        <v>1.219154344630031</v>
       </c>
       <c r="G239">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="240">
@@ -6819,10 +6819,10 @@
         <v>0.4607053674139334</v>
       </c>
       <c r="E240">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
       <c r="F240">
-        <v>0.2090120962215762</v>
+        <v>0.2102485111995552</v>
       </c>
       <c r="G240">
         <v>6</v>
@@ -6842,8 +6842,17 @@
           <t>rural_interstate_poor_percent_score</t>
         </is>
       </c>
+      <c r="D241">
+        <v>1.490372158032406</v>
+      </c>
       <c r="E241">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
+      </c>
+      <c r="F241">
+        <v>0.68014950448373</v>
+      </c>
+      <c r="G241">
+        <v>28</v>
       </c>
     </row>
     <row r="242">
@@ -6864,10 +6873,10 @@
         <v>0.3065694171628117</v>
       </c>
       <c r="E242">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
       <c r="F242">
-        <v>0.1390839374811421</v>
+        <v>0.1399066911236666</v>
       </c>
       <c r="G242">
         <v>4</v>
@@ -6891,10 +6900,10 @@
         <v>0.6388843010613818</v>
       </c>
       <c r="E243">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
       <c r="F243">
-        <v>0.2898480383622668</v>
+        <v>0.2915626398731239</v>
       </c>
       <c r="G243">
         <v>14</v>
@@ -6918,10 +6927,10 @@
         <v>1.045386045442011</v>
       </c>
       <c r="E244">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
       <c r="F244">
-        <v>0.4742691189927093</v>
+        <v>0.477074666867287</v>
       </c>
       <c r="G244">
         <v>21</v>
@@ -6945,10 +6954,10 @@
         <v>0.4820030293160084</v>
       </c>
       <c r="E245">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
       <c r="F245">
-        <v>0.218674386426178</v>
+        <v>0.219967958863206</v>
       </c>
       <c r="G245">
         <v>8</v>
@@ -6972,10 +6981,10 @@
         <v>0.9468303298836719</v>
       </c>
       <c r="E246">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
       <c r="F246">
-        <v>0.4295565148850219</v>
+        <v>0.4320975645108256</v>
       </c>
       <c r="G246">
         <v>18</v>
@@ -6999,10 +7008,10 @@
         <v>0.5443032484711802</v>
       </c>
       <c r="E247">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
       <c r="F247">
-        <v>0.2469386531825635</v>
+        <v>0.2483994234200583</v>
       </c>
       <c r="G247">
         <v>11</v>
@@ -7026,13 +7035,13 @@
         <v>4.172191935563085</v>
       </c>
       <c r="E248">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
       <c r="F248">
-        <v>1.892833563424254</v>
+        <v>1.904030655893764</v>
       </c>
       <c r="G248">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="249">
@@ -7053,13 +7062,13 @@
         <v>1.919207069381429</v>
       </c>
       <c r="E249">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
       <c r="F249">
-        <v>0.8707028852439385</v>
+        <v>0.8758535445031225</v>
       </c>
       <c r="G249">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="250">
@@ -7080,10 +7089,10 @@
         <v>1.376146788990826</v>
       </c>
       <c r="E250">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
       <c r="F250">
-        <v>0.6243281398914836</v>
+        <v>0.6280213647205253</v>
       </c>
       <c r="G250">
         <v>26</v>
@@ -7107,10 +7116,10 @@
         <v>1.430943722780659</v>
       </c>
       <c r="E251">
-        <v>2.20420432952136</v>
+        <v>2.191241996366194</v>
       </c>
       <c r="F251">
-        <v>0.6491883277860115</v>
+        <v>0.6530286135231241</v>
       </c>
       <c r="G251">
         <v>27</v>
@@ -11184,13 +11193,13 @@
         <v>3.841884334507866</v>
       </c>
       <c r="E402">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F402">
-        <v>0.8392836707650408</v>
+        <v>0.8489543281514237</v>
       </c>
       <c r="G402">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="403">
@@ -11211,13 +11220,13 @@
         <v>1.347849284788739</v>
       </c>
       <c r="E403">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F403">
-        <v>0.2944461094819594</v>
+        <v>0.2978388687393364</v>
       </c>
       <c r="G403">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="404">
@@ -11238,13 +11247,13 @@
         <v>2.726697274576115</v>
       </c>
       <c r="E404">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F404">
-        <v>0.5956640800234869</v>
+        <v>0.6025276273983944</v>
       </c>
       <c r="G404">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="405">
@@ -11265,13 +11274,13 @@
         <v>5.178207202683184</v>
       </c>
       <c r="E405">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F405">
-        <v>1.131211762419345</v>
+        <v>1.144246165168814</v>
       </c>
       <c r="G405">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="406">
@@ -11292,13 +11301,13 @@
         <v>10.15575488391877</v>
       </c>
       <c r="E406">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F406">
-        <v>2.218588196892497</v>
+        <v>2.244151909235503</v>
       </c>
       <c r="G406">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="407">
@@ -11319,13 +11328,13 @@
         <v>7.466878259495337</v>
       </c>
       <c r="E407">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F407">
-        <v>1.631186274531008</v>
+        <v>1.649981640321909</v>
       </c>
       <c r="G407">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="408">
@@ -11346,13 +11355,13 @@
         <v>1.578133383833602</v>
       </c>
       <c r="E408">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F408">
-        <v>0.3447531117592547</v>
+        <v>0.3487255341270985</v>
       </c>
       <c r="G408">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="409">
@@ -11373,13 +11382,13 @@
         <v>7.784133300174085</v>
       </c>
       <c r="E409">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F409">
-        <v>1.700492623167784</v>
+        <v>1.720086572293158</v>
       </c>
       <c r="G409">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="410">
@@ -11400,13 +11409,13 @@
         <v>1.178262761922527</v>
       </c>
       <c r="E410">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F410">
-        <v>0.2573988724933252</v>
+        <v>0.2603647544641434</v>
       </c>
       <c r="G410">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="411">
@@ -11427,13 +11436,13 @@
         <v>1.619157279245838</v>
       </c>
       <c r="E411">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F411">
-        <v>0.3537150383902588</v>
+        <v>0.3577907246782636</v>
       </c>
       <c r="G411">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="412">
@@ -11454,13 +11463,13 @@
         <v>16.35283180517326</v>
       </c>
       <c r="E412">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F412">
-        <v>3.572378424195119</v>
+        <v>3.613541202643324</v>
       </c>
       <c r="G412">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="413">
@@ -11481,13 +11490,13 @@
         <v>1.530150677638157</v>
       </c>
       <c r="E413">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F413">
-        <v>0.33427098937279</v>
+        <v>0.3381226313444309</v>
       </c>
       <c r="G413">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="414">
@@ -11508,13 +11517,13 @@
         <v>4.657768866052593</v>
       </c>
       <c r="E414">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F414">
-        <v>1.017518751505177</v>
+        <v>1.029243125006996</v>
       </c>
       <c r="G414">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="415">
@@ -11535,13 +11544,13 @@
         <v>3.045702818771048</v>
       </c>
       <c r="E415">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F415">
-        <v>0.6653528371059196</v>
+        <v>0.6730193741217584</v>
       </c>
       <c r="G415">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="416">
@@ -11562,13 +11571,13 @@
         <v>4.320012102222523</v>
       </c>
       <c r="E416">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F416">
-        <v>0.9437336731708669</v>
+        <v>0.9546078571150259</v>
       </c>
       <c r="G416">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="417">
@@ -11589,13 +11598,13 @@
         <v>2.485828216456696</v>
       </c>
       <c r="E417">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F417">
-        <v>0.5430447272084106</v>
+        <v>0.549301967382674</v>
       </c>
       <c r="G417">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="418">
@@ -11616,13 +11625,13 @@
         <v>4.770756685815098</v>
       </c>
       <c r="E418">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F418">
-        <v>1.04220164767419</v>
+        <v>1.054210430179149</v>
       </c>
       <c r="G418">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="419">
@@ -11643,13 +11652,13 @@
         <v>13.48845079546951</v>
       </c>
       <c r="E419">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F419">
-        <v>2.946636470773769</v>
+        <v>2.980589129146233</v>
       </c>
       <c r="G419">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="420">
@@ -11670,10 +11679,10 @@
         <v>0.6436781609195403</v>
       </c>
       <c r="E420">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F420">
-        <v>0.1406155216166975</v>
+        <v>0.1422357658560773</v>
       </c>
       <c r="G420">
         <v>2</v>
@@ -11697,13 +11706,13 @@
         <v>6.917465610671113</v>
       </c>
       <c r="E421">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F421">
-        <v>1.51116364383174</v>
+        <v>1.528576047245872</v>
       </c>
       <c r="G421">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="422">
@@ -11724,13 +11733,13 @@
         <v>2.559868008757386</v>
       </c>
       <c r="E422">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F422">
-        <v>0.559219183088474</v>
+        <v>0.5656627936481932</v>
       </c>
       <c r="G422">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="423">
@@ -11751,13 +11760,13 @@
         <v>6.155283854224003</v>
       </c>
       <c r="E423">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F423">
-        <v>1.34466027031906</v>
+        <v>1.360154136372099</v>
       </c>
       <c r="G423">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="424">
@@ -11778,13 +11787,13 @@
         <v>1.871311272284662</v>
       </c>
       <c r="E424">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F424">
-        <v>0.40879965584603</v>
+        <v>0.4135100553796638</v>
       </c>
       <c r="G424">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="425">
@@ -11805,13 +11814,13 @@
         <v>4.838151456579799</v>
       </c>
       <c r="E425">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F425">
-        <v>1.056924457023163</v>
+        <v>1.069102883296896</v>
       </c>
       <c r="G425">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="426">
@@ -11832,13 +11841,13 @@
         <v>3.2061503940556</v>
       </c>
       <c r="E426">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F426">
-        <v>0.700403613814797</v>
+        <v>0.7084740238767646</v>
       </c>
       <c r="G426">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="427">
@@ -11859,13 +11868,13 @@
         <v>1.832571670732686</v>
       </c>
       <c r="E427">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F427">
-        <v>0.4003367475011637</v>
+        <v>0.4049496330595513</v>
       </c>
       <c r="G427">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="428">
@@ -11886,13 +11895,13 @@
         <v>1.278326554328879</v>
       </c>
       <c r="E428">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F428">
-        <v>0.2792584340233658</v>
+        <v>0.2824761930859674</v>
       </c>
       <c r="G428">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="429">
@@ -11913,13 +11922,13 @@
         <v>2.693602693602694</v>
       </c>
       <c r="E429">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F429">
-        <v>0.5884343617437559</v>
+        <v>0.5952146045925314</v>
       </c>
       <c r="G429">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="430">
@@ -11940,10 +11949,10 @@
         <v>0.103849924397255</v>
       </c>
       <c r="E430">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F430">
-        <v>0.02268666575251414</v>
+        <v>0.02294807316382712</v>
       </c>
       <c r="G430">
         <v>1</v>
@@ -11967,13 +11976,13 @@
         <v>6.249579756305207</v>
       </c>
       <c r="E431">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F431">
-        <v>1.365259800119051</v>
+        <v>1.380991024531314</v>
       </c>
       <c r="G431">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="432">
@@ -11994,13 +12003,13 @@
         <v>4.317257834730335</v>
       </c>
       <c r="E432">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F432">
-        <v>0.9431319862043048</v>
+        <v>0.9539992372022977</v>
       </c>
       <c r="G432">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="433">
@@ -12021,13 +12030,13 @@
         <v>8.83566379056867</v>
       </c>
       <c r="E433">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F433">
-        <v>1.930206038007687</v>
+        <v>1.952446863045644</v>
       </c>
       <c r="G433">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="434">
@@ -12048,13 +12057,13 @@
         <v>2.715116558645373</v>
       </c>
       <c r="E434">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F434">
-        <v>0.5931342001702233</v>
+        <v>0.5999685969704898</v>
       </c>
       <c r="G434">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="435">
@@ -12075,10 +12084,10 @@
         <v>0.6535040067964417</v>
       </c>
       <c r="E435">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F435">
-        <v>0.1427620391268333</v>
+        <v>0.1444070166430984</v>
       </c>
       <c r="G435">
         <v>3</v>
@@ -12102,13 +12111,13 @@
         <v>2.982166541645014</v>
       </c>
       <c r="E436">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F436">
-        <v>0.6514729398341261</v>
+        <v>0.658979545546939</v>
       </c>
       <c r="G436">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="437">
@@ -12129,13 +12138,13 @@
         <v>5.636682543164782</v>
       </c>
       <c r="E437">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F437">
-        <v>1.231368569134855</v>
+        <v>1.245557030037006</v>
       </c>
       <c r="G437">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="438">
@@ -12156,13 +12165,13 @@
         <v>2.48751973375432</v>
       </c>
       <c r="E438">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F438">
-        <v>0.5434142497455575</v>
+        <v>0.5496757477482259</v>
       </c>
       <c r="G438">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="439">
@@ -12183,13 +12192,13 @@
         <v>5.686412198425039</v>
       </c>
       <c r="E439">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F439">
-        <v>1.242232323474834</v>
+        <v>1.256545962132506</v>
       </c>
       <c r="G439">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="440">
@@ -12210,13 +12219,13 @@
         <v>1.561008155893755</v>
       </c>
       <c r="E440">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F440">
-        <v>0.3410119985667141</v>
+        <v>0.3449413139074716</v>
       </c>
       <c r="G440">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="441">
@@ -12233,8 +12242,17 @@
           <t>urban_interstate_poor_percent_score</t>
         </is>
       </c>
+      <c r="D441">
+        <v>1.11074743901335</v>
+      </c>
       <c r="E441">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
+      </c>
+      <c r="F441">
+        <v>0.2454456625265073</v>
+      </c>
+      <c r="G441">
+        <v>5</v>
       </c>
     </row>
     <row r="442">
@@ -12255,13 +12273,13 @@
         <v>1.5954597773194</v>
       </c>
       <c r="E442">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F442">
-        <v>0.3485381708239607</v>
+        <v>0.3525542065857939</v>
       </c>
       <c r="G442">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="443">
@@ -12282,13 +12300,13 @@
         <v>1.592308278328465</v>
       </c>
       <c r="E443">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F443">
-        <v>0.3478497061511003</v>
+        <v>0.3518578090694793</v>
       </c>
       <c r="G443">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="444">
@@ -12309,13 +12327,13 @@
         <v>4.518636501668191</v>
       </c>
       <c r="E444">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F444">
-        <v>0.9871244159823931</v>
+        <v>0.9984985703442875</v>
       </c>
       <c r="G444">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="445">
@@ -12336,13 +12354,13 @@
         <v>2.367643780101138</v>
       </c>
       <c r="E445">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F445">
-        <v>0.5172265976304684</v>
+        <v>0.523186348059366</v>
       </c>
       <c r="G445">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="446">
@@ -12363,10 +12381,10 @@
         <v>0.7491278345377524</v>
       </c>
       <c r="E446">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F446">
-        <v>0.1636516625958365</v>
+        <v>0.1655373410795291</v>
       </c>
       <c r="G446">
         <v>4</v>
@@ -12390,13 +12408,13 @@
         <v>2.685387422313179</v>
       </c>
       <c r="E447">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F447">
-        <v>0.5866396843292735</v>
+        <v>0.5933992479833987</v>
       </c>
       <c r="G447">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="448">
@@ -12417,13 +12435,13 @@
         <v>3.654223968565815</v>
       </c>
       <c r="E448">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F448">
-        <v>0.7982880896721158</v>
+        <v>0.8074863749238854</v>
       </c>
       <c r="G448">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="449">
@@ -12444,13 +12462,13 @@
         <v>3.768761269459659</v>
       </c>
       <c r="E449">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F449">
-        <v>0.8233094796890589</v>
+        <v>0.8327960742438848</v>
       </c>
       <c r="G449">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="450">
@@ -12471,13 +12489,13 @@
         <v>4.704226906522459</v>
       </c>
       <c r="E450">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F450">
-        <v>1.027667801124365</v>
+        <v>1.039509117186945</v>
       </c>
       <c r="G450">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="451">
@@ -12498,13 +12516,13 @@
         <v>7.453510802834312</v>
       </c>
       <c r="E451">
-        <v>4.577575459088623</v>
+        <v>4.525431118153872</v>
       </c>
       <c r="F451">
-        <v>1.628266069985939</v>
+        <v>1.647027787680688</v>
       </c>
       <c r="G451">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="452">
@@ -19030,10 +19048,10 @@
         <v>5</v>
       </c>
       <c r="H2">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="I2">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="J2">
         <v>5</v>
@@ -19082,10 +19100,10 @@
         <v>28</v>
       </c>
       <c r="H3">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I3">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J3">
         <v>50</v>
@@ -19134,10 +19152,10 @@
         <v>36</v>
       </c>
       <c r="H4">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I4">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J4">
         <v>42</v>
@@ -19186,10 +19204,10 @@
         <v>26</v>
       </c>
       <c r="H5">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="I5">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="J5">
         <v>25</v>
@@ -19238,10 +19256,10 @@
         <v>48</v>
       </c>
       <c r="H6">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I6">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J6">
         <v>39</v>
@@ -19290,10 +19308,10 @@
         <v>18</v>
       </c>
       <c r="H7">
+        <v>46</v>
+      </c>
+      <c r="I7">
         <v>45</v>
-      </c>
-      <c r="I7">
-        <v>44</v>
       </c>
       <c r="J7">
         <v>33</v>
@@ -19345,7 +19363,7 @@
         <v>1</v>
       </c>
       <c r="I8">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J8">
         <v>32</v>
@@ -19394,7 +19412,7 @@
         <v>23</v>
       </c>
       <c r="I9">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="J9">
         <v>6</v>
@@ -19446,7 +19464,7 @@
         <v>2</v>
       </c>
       <c r="I10">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J10">
         <v>7</v>
@@ -19498,7 +19516,7 @@
         <v>16</v>
       </c>
       <c r="I11">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J11">
         <v>3</v>
@@ -19532,7 +19550,7 @@
         </is>
       </c>
       <c r="C12">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D12">
         <v>9</v>
@@ -19547,7 +19565,7 @@
         <v>6</v>
       </c>
       <c r="I12">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J12">
         <v>48</v>
@@ -19599,7 +19617,7 @@
         <v>22</v>
       </c>
       <c r="I13">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J13">
         <v>19</v>
@@ -19651,7 +19669,7 @@
         <v>25</v>
       </c>
       <c r="I14">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="J14">
         <v>46</v>
@@ -19685,7 +19703,7 @@
         </is>
       </c>
       <c r="C15">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D15">
         <v>46</v>
@@ -19700,10 +19718,10 @@
         <v>3</v>
       </c>
       <c r="H15">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="I15">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="J15">
         <v>4</v>
@@ -19752,10 +19770,10 @@
         <v>19</v>
       </c>
       <c r="H16">
+        <v>33</v>
+      </c>
+      <c r="I16">
         <v>32</v>
-      </c>
-      <c r="I16">
-        <v>31</v>
       </c>
       <c r="J16">
         <v>38</v>
@@ -19807,7 +19825,7 @@
         <v>13</v>
       </c>
       <c r="I17">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J17">
         <v>8</v>
@@ -19859,7 +19877,7 @@
         <v>24</v>
       </c>
       <c r="I18">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J18">
         <v>15</v>
@@ -19908,10 +19926,10 @@
         <v>33</v>
       </c>
       <c r="H19">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="I19">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="J19">
         <v>47</v>
@@ -20012,10 +20030,10 @@
         <v>42</v>
       </c>
       <c r="H21">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="I21">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J21">
         <v>30</v>
@@ -20049,7 +20067,7 @@
         </is>
       </c>
       <c r="C22">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D22">
         <v>6</v>
@@ -20064,10 +20082,10 @@
         <v>10</v>
       </c>
       <c r="H22">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="I22">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J22">
         <v>17</v>
@@ -20116,10 +20134,10 @@
         <v>21</v>
       </c>
       <c r="H23">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="I23">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="J23">
         <v>16</v>
@@ -20171,7 +20189,7 @@
         <v>9</v>
       </c>
       <c r="I24">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J24">
         <v>22</v>
@@ -20220,10 +20238,10 @@
         <v>12</v>
       </c>
       <c r="H25">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="I25">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="J25">
         <v>34</v>
@@ -20275,7 +20293,7 @@
         <v>23</v>
       </c>
       <c r="I26">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="J26">
         <v>13</v>
@@ -20324,10 +20342,10 @@
         <v>30</v>
       </c>
       <c r="H27">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="I27">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="J27">
         <v>26</v>
@@ -20379,7 +20397,7 @@
         <v>12</v>
       </c>
       <c r="I28">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J28">
         <v>44</v>
@@ -20431,7 +20449,7 @@
         <v>10</v>
       </c>
       <c r="I29">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="J29">
         <v>2</v>
@@ -20535,7 +20553,7 @@
         <v>17</v>
       </c>
       <c r="I31">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="J31">
         <v>31</v>
@@ -20584,10 +20602,10 @@
         <v>31</v>
       </c>
       <c r="H32">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="I32">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="J32">
         <v>35</v>
@@ -20636,10 +20654,10 @@
         <v>49</v>
       </c>
       <c r="H33">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="I33">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J33">
         <v>28</v>
@@ -20673,7 +20691,7 @@
         </is>
       </c>
       <c r="C34">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D34">
         <v>8</v>
@@ -20691,7 +20709,7 @@
         <v>20</v>
       </c>
       <c r="I34">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="J34">
         <v>20</v>
@@ -20777,7 +20795,7 @@
         </is>
       </c>
       <c r="C36">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D36">
         <v>10</v>
@@ -20795,7 +20813,7 @@
         <v>19</v>
       </c>
       <c r="I36">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J36">
         <v>9</v>
@@ -20844,10 +20862,10 @@
         <v>44</v>
       </c>
       <c r="H37">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I37">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="J37">
         <v>45</v>
@@ -20899,7 +20917,7 @@
         <v>15</v>
       </c>
       <c r="I38">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J38">
         <v>24</v>
@@ -20948,10 +20966,10 @@
         <v>39</v>
       </c>
       <c r="H39">
+        <v>41</v>
+      </c>
+      <c r="I39">
         <v>40</v>
-      </c>
-      <c r="I39">
-        <v>39</v>
       </c>
       <c r="J39">
         <v>37</v>
@@ -20985,7 +21003,7 @@
         </is>
       </c>
       <c r="C40">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D40">
         <v>31</v>
@@ -21003,7 +21021,7 @@
         <v>6</v>
       </c>
       <c r="I40">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J40">
         <v>49</v>
@@ -21037,7 +21055,7 @@
         </is>
       </c>
       <c r="C41">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D41">
         <v>1</v>
@@ -21051,6 +21069,12 @@
       <c r="G41">
         <v>1</v>
       </c>
+      <c r="H41">
+        <v>28</v>
+      </c>
+      <c r="I41">
+        <v>5</v>
+      </c>
       <c r="J41">
         <v>21</v>
       </c>
@@ -21101,7 +21125,7 @@
         <v>4</v>
       </c>
       <c r="I42">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J42">
         <v>18</v>
@@ -21153,7 +21177,7 @@
         <v>14</v>
       </c>
       <c r="I43">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J43">
         <v>27</v>
@@ -21205,7 +21229,7 @@
         <v>21</v>
       </c>
       <c r="I44">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="J44">
         <v>12</v>
@@ -21257,7 +21281,7 @@
         <v>8</v>
       </c>
       <c r="I45">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J45">
         <v>10</v>
@@ -21361,7 +21385,7 @@
         <v>11</v>
       </c>
       <c r="I47">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J47">
         <v>11</v>
@@ -21410,10 +21434,10 @@
         <v>50</v>
       </c>
       <c r="H48">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="I48">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J48">
         <v>29</v>
@@ -21462,10 +21486,10 @@
         <v>8</v>
       </c>
       <c r="H49">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="I49">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J49">
         <v>36</v>
@@ -21517,7 +21541,7 @@
         <v>26</v>
       </c>
       <c r="I50">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="J50">
         <v>40</v>
@@ -21569,7 +21593,7 @@
         <v>27</v>
       </c>
       <c r="I51">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="J51">
         <v>1</v>

</xml_diff>